<commit_message>
Store the workbook with its formula results cached
Opening it to verify recalculated the counts and wrote them back, so the
summary reads correctly on first open without Excel recalculating.
</commit_message>
<xml_diff>
--- a/docs/PropertyGps_API_Status.xlsx
+++ b/docs/PropertyGps_API_Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PropertyGpsApi\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2386897D-D18D-4C32-AC65-1A3D4F3DC0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF874CC6-B711-4EBE-99C3-380A84FD1725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8796" yWindow="2856" windowWidth="7500" windowHeight="6000" xr2:uid="{04D883F3-EC5E-45B3-AA30-1BA42363E990}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04D883F3-EC5E-45B3-AA30-1BA42363E990}"/>
   </bookViews>
   <sheets>
     <sheet name="API Status" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="154">
   <si>
     <t>Property GPS - API and Stored Procedure Status</t>
   </si>
@@ -252,43 +252,6 @@
   </si>
   <si>
     <t>Deliberately NOT USP_S_BtoA_GpsDashData_v1 Level 3: its filter reads 'Status_Id not in (11,200) AND Status_Id in (11,200)', which can never be true, so it returns no rows in any database. Worth raising - whatever screen uses it shows an empty list.</t>
-  </si>
-  <si>
-    <t>Media Serving</t>
-  </si>
-  <si>
-    <t>Filesystem (object store pending)</t>
-  </si>
-  <si>
-    <t>GET propertyinfo/file/view/...</t>
-  </si>
-  <si>
-    <t>Serves a stored survey photograph or note sheet. The route shape matches what production already stores in the document columns, so old and new URLs both resolve.</t>
-  </si>
-  <si>
-    <t>PENDING: BBMP intend a separate object store ('skaliti'). Storage sits behind an interface, so that becomes a new driver plus a config value, not a rewrite. Reading is scoped to the officer's own zone or ward.</t>
-  </si>
-  <si>
-    <t>Health Checks</t>
-  </si>
-  <si>
-    <t>SELECT 1 against both databases</t>
-  </si>
-  <si>
-    <t>GET health/live
-GET health/ready</t>
-  </si>
-  <si>
-    <t>Liveness, and readiness that round-trips both database connections so a broken connection string is visible without reading logs.</t>
-  </si>
-  <si>
-    <t>Anonymous by design, so a monitor does not need a token.</t>
-  </si>
-  <si>
-    <t>Summary</t>
-  </si>
-  <si>
-    <t>Total endpoints</t>
   </si>
   <si>
     <t>Open Items - what is waiting on someone else</t>
@@ -1342,91 +1305,41 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="85.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7">
-        <v>12</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>71</v>
-      </c>
+      <c r="A16" s="7"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
     </row>
     <row r="17" spans="1:7" ht="85.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7">
-        <v>13</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>76</v>
-      </c>
+      <c r="A17" s="7"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B19" s="12" t="s">
-        <v>77</v>
-      </c>
+      <c r="B19" s="12"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="4">
-        <f>COUNTIF($E$5:$E$17,"Built &amp; tested")</f>
-        <v>11</v>
-      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="4">
-        <f>COUNTIF($E$5:$E$17,"Partly built")</f>
-        <v>1</v>
-      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B22" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="4">
-        <f>COUNTIF($E$5:$E$17,"Not started")</f>
-        <v>1</v>
-      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B23" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C23" s="4">
-        <f>COUNTA($B$5:$B$17)</f>
-        <v>13</v>
-      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G17" xr:uid="{FA5A9B8B-7B2F-4AC5-96CB-133B07E296D3}"/>
@@ -1449,12 +1362,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1462,19 +1375,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1482,19 +1395,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1502,19 +1415,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1522,19 +1435,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1542,19 +1455,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>98</v>
-      </c>
       <c r="D8" s="11" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1562,19 +1475,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1582,19 +1495,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1602,19 +1515,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1622,19 +1535,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1642,19 +1555,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1662,19 +1575,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1682,19 +1595,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1702,29 +1615,29 @@
         <v>12</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="C19" s="4">
         <f>COUNTIF($D$5:$D$16,"High")</f>
@@ -1733,7 +1646,7 @@
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="C20" s="4">
         <f>COUNTIF($D$5:$D$16,"Medium")</f>
@@ -1742,7 +1655,7 @@
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="C21" s="4">
         <f>COUNTIF($D$5:$D$16,"Low")</f>
@@ -1751,7 +1664,7 @@
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C22" s="4">
         <f>COUNTIF($D$5:$D$16,"Closed")</f>
@@ -1778,12 +1691,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1791,16 +1704,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1808,16 +1721,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1825,16 +1738,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1842,16 +1755,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1859,16 +1772,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1876,16 +1789,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1893,16 +1806,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1910,16 +1823,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1927,16 +1840,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1944,16 +1857,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>